<commit_message>
Update tutorial and locales
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fengmingliu/Dev/ProjectMT3/Data/Locale/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0263CEDC-C360-5349-8E90-8F4B555C1DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C372DBD2-842F-8A4D-8653-24A5171CC3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" firstSheet="1" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="1417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="1504">
   <si>
     <t>ID</t>
   </si>
@@ -3728,12 +3728,6 @@
     <t>TM_05</t>
   </si>
   <si>
-    <t>敌人的能力信息，确认键或点击可以查看详细内容。</t>
-  </si>
-  <si>
-    <t>There is the information of enemies. You can press confirm button or click to view the detail.</t>
-  </si>
-  <si>
     <t>TMT3_001</t>
   </si>
   <si>
@@ -4010,21 +4004,6 @@
     <t>TM_07</t>
   </si>
   <si>
-    <t>按 B 键可以快速使用，在这里可以查看更多快捷键。</t>
-  </si>
-  <si>
-    <t>You can use them quickly by pressing B. Here you can view more of hotkeys.</t>
-  </si>
-  <si>
-    <t>TM_08</t>
-  </si>
-  <si>
-    <t>You can use them quickly by pressing N. Here you can view more of hotkeys.</t>
-  </si>
-  <si>
-    <t>按 N 键可以快速使用，在这里可以查看更多快捷键。</t>
-  </si>
-  <si>
     <t>玩家每次移动后，若处于敌人的{value}格范围内，敌人造成一次单回合伤害。</t>
   </si>
   <si>
@@ -4296,6 +4275,288 @@
   </si>
   <si>
     <t>巧妙运用手中道具，不必与强敌作战就可前进。</t>
+  </si>
+  <si>
+    <t>Slime</t>
+  </si>
+  <si>
+    <t>Red Slime</t>
+  </si>
+  <si>
+    <t>Bat</t>
+  </si>
+  <si>
+    <t>Water Mage</t>
+  </si>
+  <si>
+    <t>Guard</t>
+  </si>
+  <si>
+    <t>Thunder Mage</t>
+  </si>
+  <si>
+    <t>Skeleton</t>
+  </si>
+  <si>
+    <t>Black Slime</t>
+  </si>
+  <si>
+    <t>Slime Man</t>
+  </si>
+  <si>
+    <t>Zombie</t>
+  </si>
+  <si>
+    <t>Big Bat</t>
+  </si>
+  <si>
+    <t>Stone Golem</t>
+  </si>
+  <si>
+    <t>Knight</t>
+  </si>
+  <si>
+    <t>Greatsword Fighter</t>
+  </si>
+  <si>
+    <t>Skeleton Soldier</t>
+  </si>
+  <si>
+    <t>Skeleton Armiger</t>
+  </si>
+  <si>
+    <t>Veteran Guard</t>
+  </si>
+  <si>
+    <t>Iron Knight</t>
+  </si>
+  <si>
+    <t>Red Bat</t>
+  </si>
+  <si>
+    <t>Baby Octopus</t>
+  </si>
+  <si>
+    <t>Slime Berserker</t>
+  </si>
+  <si>
+    <t>Slime King</t>
+  </si>
+  <si>
+    <t>Flame Mage</t>
+  </si>
+  <si>
+    <t>Zombie Swordsman</t>
+  </si>
+  <si>
+    <t>Archer</t>
+  </si>
+  <si>
+    <t>Demon Slime</t>
+  </si>
+  <si>
+    <t>Blood Bat</t>
+  </si>
+  <si>
+    <t>Skeleton Captain</t>
+  </si>
+  <si>
+    <t>Wind Wizard</t>
+  </si>
+  <si>
+    <t>Evil-Eye Slime</t>
+  </si>
+  <si>
+    <t>White Guard</t>
+  </si>
+  <si>
+    <t>Grey Knight</t>
+  </si>
+  <si>
+    <t>Nether Mage</t>
+  </si>
+  <si>
+    <t>Big Slime</t>
+  </si>
+  <si>
+    <t>Mage</t>
+  </si>
+  <si>
+    <t>Poison Zombie</t>
+  </si>
+  <si>
+    <t>Poison Bat</t>
+  </si>
+  <si>
+    <t>Skeleton Chief</t>
+  </si>
+  <si>
+    <t>Conehead</t>
+  </si>
+  <si>
+    <t>Orc</t>
+  </si>
+  <si>
+    <t>Crab Slime</t>
+  </si>
+  <si>
+    <t>Elite Archer</t>
+  </si>
+  <si>
+    <t>Frail Sentinel</t>
+  </si>
+  <si>
+    <t>Berserk Sentinel</t>
+  </si>
+  <si>
+    <t>Speedster</t>
+  </si>
+  <si>
+    <t>Blue Guard</t>
+  </si>
+  <si>
+    <t>Demon Guard</t>
+  </si>
+  <si>
+    <t>Swift Hound</t>
+  </si>
+  <si>
+    <t>Steel Golem</t>
+  </si>
+  <si>
+    <t>Elite Guard</t>
+  </si>
+  <si>
+    <t>Iron Golem</t>
+  </si>
+  <si>
+    <t>Mercury Man</t>
+  </si>
+  <si>
+    <t>Adept Mage</t>
+  </si>
+  <si>
+    <t>Unstable Machine</t>
+  </si>
+  <si>
+    <t>Armoured Skeleton</t>
+  </si>
+  <si>
+    <t>Medium Bat</t>
+  </si>
+  <si>
+    <t>Ice Slime</t>
+  </si>
+  <si>
+    <t>Poison Octopus</t>
+  </si>
+  <si>
+    <t>Blazing Zombie</t>
+  </si>
+  <si>
+    <t>Frozen Bones</t>
+  </si>
+  <si>
+    <t>Sentinel</t>
+  </si>
+  <si>
+    <t>Ironclad Sentinel</t>
+  </si>
+  <si>
+    <t>Royal Knight</t>
+  </si>
+  <si>
+    <t>Ghost Flame</t>
+  </si>
+  <si>
+    <t>Orc Soldier</t>
+  </si>
+  <si>
+    <t>Flame Wizard</t>
+  </si>
+  <si>
+    <t>Crimson Overlord</t>
+  </si>
+  <si>
+    <t>Vampire Count</t>
+  </si>
+  <si>
+    <t>Hammer Skeleton</t>
+  </si>
+  <si>
+    <t>Gale Hound</t>
+  </si>
+  <si>
+    <t>Giant Bat</t>
+  </si>
+  <si>
+    <t>Frail Octopus</t>
+  </si>
+  <si>
+    <t>Frost Wizard</t>
+  </si>
+  <si>
+    <t>Tentacle Plant</t>
+  </si>
+  <si>
+    <t>Archmage</t>
+  </si>
+  <si>
+    <t>Skeleton Swordsman</t>
+  </si>
+  <si>
+    <t>Giant Octopus</t>
+  </si>
+  <si>
+    <t>Demon Dragon</t>
+  </si>
+  <si>
+    <t>Death Knight</t>
+  </si>
+  <si>
+    <t>Blood Mage</t>
+  </si>
+  <si>
+    <t>Slime Asura</t>
+  </si>
+  <si>
+    <t>Mad Tentacle</t>
+  </si>
+  <si>
+    <t>Royal Lancer</t>
+  </si>
+  <si>
+    <t>Dragon Bat</t>
+  </si>
+  <si>
+    <t>敌人的能力信息，确认键查看详细内容。</t>
+  </si>
+  <si>
+    <t>There is the information of enemies. You can press confirm button to view the detail.</t>
+  </si>
+  <si>
+    <t>TM_05_M</t>
+  </si>
+  <si>
+    <t>There is the information of enemies. You can click to view the detail.</t>
+  </si>
+  <si>
+    <t>敌人的能力信息，点击查看详细内容。</t>
+  </si>
+  <si>
+    <t>按 N 键可以快速使用。</t>
+  </si>
+  <si>
+    <t>You can use them quickly by pressing N.</t>
+  </si>
+  <si>
+    <t>拾取血瓶时，溢出的HP会储存在你的背包中。按 B 键可以快速使用。</t>
+  </si>
+  <si>
+    <t>When picking up a potion, any excess HP is stored in your inventory.You can use them quickly by pressing B.</t>
+  </si>
+  <si>
+    <t>TM_06_D</t>
   </si>
 </sst>
 </file>
@@ -5334,134 +5595,134 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
+        <v>1254</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C65" t="s">
         <v>1256</v>
-      </c>
-      <c r="B65" t="s">
-        <v>1257</v>
-      </c>
-      <c r="C65" t="s">
-        <v>1258</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B68" t="s">
+        <v>1260</v>
+      </c>
+      <c r="C68" t="s">
         <v>1261</v>
-      </c>
-      <c r="B68" t="s">
-        <v>1262</v>
-      </c>
-      <c r="C68" t="s">
-        <v>1263</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B69" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C69" t="s">
         <v>1264</v>
-      </c>
-      <c r="B69" t="s">
-        <v>1265</v>
-      </c>
-      <c r="C69" t="s">
-        <v>1266</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B70" t="s">
+        <v>1266</v>
+      </c>
+      <c r="C70" t="s">
         <v>1267</v>
-      </c>
-      <c r="B70" t="s">
-        <v>1268</v>
-      </c>
-      <c r="C70" t="s">
-        <v>1269</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B71" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C71" t="s">
         <v>1270</v>
-      </c>
-      <c r="B71" t="s">
-        <v>1271</v>
-      </c>
-      <c r="C71" t="s">
-        <v>1272</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B72" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C72" t="s">
         <v>1273</v>
-      </c>
-      <c r="B72" t="s">
-        <v>1274</v>
-      </c>
-      <c r="C72" t="s">
-        <v>1275</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B73" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C73" t="s">
         <v>1276</v>
-      </c>
-      <c r="B73" t="s">
-        <v>1277</v>
-      </c>
-      <c r="C73" t="s">
-        <v>1278</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>1282</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>1299</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B76" t="s">
+        <v>1312</v>
+      </c>
+      <c r="C76" t="s">
         <v>1313</v>
-      </c>
-      <c r="B76" t="s">
-        <v>1314</v>
-      </c>
-      <c r="C76" t="s">
-        <v>1315</v>
       </c>
     </row>
   </sheetData>
@@ -5660,10 +5921,10 @@
         <v>966</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1327</v>
+        <v>1320</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1326</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -5803,7 +6064,7 @@
         <v>1003</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
       <c r="C30" t="s">
         <v>1004</v>
@@ -5814,7 +6075,7 @@
         <v>1005</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="C31" t="s">
         <v>1006</v>
@@ -6426,7 +6687,7 @@
         <v>16</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1328</v>
+        <v>1321</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>1206</v>
@@ -6437,7 +6698,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1329</v>
+        <v>1322</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>1227</v>
@@ -6459,7 +6720,7 @@
         <v>19</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1330</v>
+        <v>1323</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>1209</v>
@@ -6481,10 +6742,10 @@
         <v>21</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -6492,10 +6753,10 @@
         <v>22</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1289</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -6503,10 +6764,10 @@
         <v>23</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>1331</v>
+        <v>1324</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -6525,10 +6786,10 @@
         <v>26</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>1332</v>
+        <v>1325</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -6536,10 +6797,10 @@
         <v>27</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1333</v>
+        <v>1326</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -6547,10 +6808,10 @@
         <v>28</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>1334</v>
+        <v>1327</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>1382</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -6558,10 +6819,10 @@
         <v>29</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1380</v>
+        <v>1373</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1381</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -6569,10 +6830,10 @@
         <v>30</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>1335</v>
+        <v>1328</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>1383</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -6580,10 +6841,10 @@
         <v>31</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>1336</v>
+        <v>1329</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1384</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -6591,10 +6852,10 @@
         <v>32</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>1337</v>
+        <v>1330</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1385</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -6602,10 +6863,10 @@
         <v>33</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>1338</v>
+        <v>1331</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1386</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -6613,10 +6874,10 @@
         <v>34</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1388</v>
+        <v>1381</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>1387</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -6624,10 +6885,10 @@
         <v>35</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>1339</v>
+        <v>1332</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1389</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -6635,7 +6896,7 @@
         <v>36</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>1340</v>
+        <v>1333</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>37</v>
@@ -6646,10 +6907,10 @@
         <v>38</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1341</v>
+        <v>1334</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1390</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -6657,10 +6918,10 @@
         <v>39</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>1342</v>
+        <v>1335</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>1391</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -6668,10 +6929,10 @@
         <v>40</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>1343</v>
+        <v>1336</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1392</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -6679,10 +6940,10 @@
         <v>41</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>1344</v>
+        <v>1337</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>1393</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -6690,10 +6951,10 @@
         <v>42</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>1345</v>
+        <v>1338</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1394</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -6701,10 +6962,10 @@
         <v>43</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>1346</v>
+        <v>1339</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>1395</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -6712,7 +6973,7 @@
         <v>44</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>1347</v>
+        <v>1340</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>45</v>
@@ -6723,7 +6984,7 @@
         <v>46</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>1378</v>
+        <v>1371</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>47</v>
@@ -6734,7 +6995,7 @@
         <v>48</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>1348</v>
+        <v>1341</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>49</v>
@@ -6745,7 +7006,7 @@
         <v>50</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>1349</v>
+        <v>1342</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>51</v>
@@ -6756,7 +7017,7 @@
         <v>52</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1377</v>
+        <v>1370</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>53</v>
@@ -6767,10 +7028,10 @@
         <v>54</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>1350</v>
+        <v>1343</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>1397</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -6778,7 +7039,7 @@
         <v>55</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>1351</v>
+        <v>1344</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>56</v>
@@ -6789,10 +7050,10 @@
         <v>57</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>1352</v>
+        <v>1345</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>1398</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -6800,10 +7061,10 @@
         <v>58</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1379</v>
+        <v>1372</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>1396</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -6811,7 +7072,7 @@
         <v>59</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>1353</v>
+        <v>1346</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>60</v>
@@ -6822,10 +7083,10 @@
         <v>61</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>1354</v>
+        <v>1347</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>1399</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -6833,10 +7094,10 @@
         <v>62</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>1355</v>
+        <v>1348</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>1400</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -6844,10 +7105,10 @@
         <v>63</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>1356</v>
+        <v>1349</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>1401</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -6855,10 +7116,10 @@
         <v>64</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>1357</v>
+        <v>1350</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>1402</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -6866,7 +7127,7 @@
         <v>65</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>1358</v>
+        <v>1351</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>66</v>
@@ -6877,10 +7138,10 @@
         <v>67</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>1359</v>
+        <v>1352</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>1403</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -6888,7 +7149,7 @@
         <v>68</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>1360</v>
+        <v>1353</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>69</v>
@@ -6899,10 +7160,10 @@
         <v>70</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>1361</v>
+        <v>1354</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>1404</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -6910,10 +7171,10 @@
         <v>71</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>1362</v>
+        <v>1355</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>1405</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -6921,7 +7182,7 @@
         <v>72</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>1363</v>
+        <v>1356</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>73</v>
@@ -6932,10 +7193,10 @@
         <v>74</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>1364</v>
+        <v>1357</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>1406</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -6943,10 +7204,10 @@
         <v>75</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>1365</v>
+        <v>1358</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>1407</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -6954,10 +7215,10 @@
         <v>76</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>1366</v>
+        <v>1359</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>1408</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -6965,10 +7226,10 @@
         <v>77</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>1367</v>
+        <v>1360</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>1409</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -6976,10 +7237,10 @@
         <v>78</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>1368</v>
+        <v>1361</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>1410</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -6987,10 +7248,10 @@
         <v>79</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>1369</v>
+        <v>1362</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>1411</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -6998,10 +7259,10 @@
         <v>80</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>1370</v>
+        <v>1363</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>1412</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -7009,10 +7270,10 @@
         <v>81</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>1371</v>
+        <v>1364</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>1413</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -7020,10 +7281,10 @@
         <v>82</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>1372</v>
+        <v>1365</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>1414</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -7031,7 +7292,7 @@
         <v>1096</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>1373</v>
+        <v>1366</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>1097</v>
@@ -7042,10 +7303,10 @@
         <v>1098</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>1374</v>
+        <v>1367</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>1415</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -7053,10 +7314,10 @@
         <v>1099</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>1375</v>
+        <v>1368</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>1416</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -7064,7 +7325,7 @@
         <v>1100</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>1376</v>
+        <v>1369</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>1101</v>
@@ -7654,7 +7915,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4933D5-C722-C646-96A3-51CA5B4C6607}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="43" customWidth="1"/>
@@ -7699,7 +7960,7 @@
         <v>1200</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>1201</v>
@@ -7710,10 +7971,10 @@
         <v>1212</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -7721,43 +7982,54 @@
         <v>1228</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1230</v>
+        <v>1495</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1229</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>1309</v>
+        <v>1496</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1311</v>
+        <v>1497</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>1310</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>1320</v>
+        <v>1307</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1322</v>
+        <v>1309</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1321</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>1323</v>
+        <v>1503</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1324</v>
+        <v>1502</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>1325</v>
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>1499</v>
       </c>
     </row>
   </sheetData>
@@ -7886,7 +8158,7 @@
         <v>284</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>286</v>
@@ -8526,46 +8798,46 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1307</v>
+        <v>1305</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1308</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>1304</v>
+        <v>1302</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
     </row>
   </sheetData>
@@ -8599,6 +8871,9 @@
       <c r="A2" t="s">
         <v>458</v>
       </c>
+      <c r="B2" t="s">
+        <v>1410</v>
+      </c>
       <c r="C2" t="s">
         <v>453</v>
       </c>
@@ -8615,6 +8890,9 @@
       <c r="A4" t="s">
         <v>460</v>
       </c>
+      <c r="B4" t="s">
+        <v>1411</v>
+      </c>
       <c r="C4" t="s">
         <v>461</v>
       </c>
@@ -8631,6 +8909,9 @@
       <c r="A6" t="s">
         <v>464</v>
       </c>
+      <c r="B6" t="s">
+        <v>1412</v>
+      </c>
       <c r="C6" t="s">
         <v>465</v>
       </c>
@@ -8647,6 +8928,9 @@
       <c r="A8" t="s">
         <v>468</v>
       </c>
+      <c r="B8" t="s">
+        <v>1413</v>
+      </c>
       <c r="C8" t="s">
         <v>469</v>
       </c>
@@ -8663,6 +8947,9 @@
       <c r="A10" t="s">
         <v>472</v>
       </c>
+      <c r="B10" t="s">
+        <v>1414</v>
+      </c>
       <c r="C10" t="s">
         <v>473</v>
       </c>
@@ -8679,6 +8966,9 @@
       <c r="A12" t="s">
         <v>476</v>
       </c>
+      <c r="B12" t="s">
+        <v>1415</v>
+      </c>
       <c r="C12" t="s">
         <v>477</v>
       </c>
@@ -8695,6 +8985,9 @@
       <c r="A14" t="s">
         <v>480</v>
       </c>
+      <c r="B14" t="s">
+        <v>1416</v>
+      </c>
       <c r="C14" t="s">
         <v>481</v>
       </c>
@@ -8711,6 +9004,9 @@
       <c r="A16" t="s">
         <v>483</v>
       </c>
+      <c r="B16" t="s">
+        <v>1417</v>
+      </c>
       <c r="C16" t="s">
         <v>484</v>
       </c>
@@ -8727,6 +9023,9 @@
       <c r="A18" t="s">
         <v>487</v>
       </c>
+      <c r="B18" t="s">
+        <v>1418</v>
+      </c>
       <c r="C18" t="s">
         <v>488</v>
       </c>
@@ -8743,6 +9042,9 @@
       <c r="A20" t="s">
         <v>491</v>
       </c>
+      <c r="B20" t="s">
+        <v>1419</v>
+      </c>
       <c r="C20" t="s">
         <v>492</v>
       </c>
@@ -8759,6 +9061,9 @@
       <c r="A22" t="s">
         <v>495</v>
       </c>
+      <c r="B22" t="s">
+        <v>1420</v>
+      </c>
       <c r="C22" t="s">
         <v>455</v>
       </c>
@@ -8775,6 +9080,9 @@
       <c r="A24" t="s">
         <v>497</v>
       </c>
+      <c r="B24" t="s">
+        <v>1421</v>
+      </c>
       <c r="C24" t="s">
         <v>498</v>
       </c>
@@ -8791,6 +9099,9 @@
       <c r="A26" t="s">
         <v>501</v>
       </c>
+      <c r="B26" t="s">
+        <v>1422</v>
+      </c>
       <c r="C26" t="s">
         <v>457</v>
       </c>
@@ -8807,6 +9118,9 @@
       <c r="A28" t="s">
         <v>504</v>
       </c>
+      <c r="B28" t="s">
+        <v>1423</v>
+      </c>
       <c r="C28" t="s">
         <v>505</v>
       </c>
@@ -8823,6 +9137,9 @@
       <c r="A30" t="s">
         <v>508</v>
       </c>
+      <c r="B30" t="s">
+        <v>1424</v>
+      </c>
       <c r="C30" t="s">
         <v>451</v>
       </c>
@@ -8839,6 +9156,9 @@
       <c r="A32" t="s">
         <v>511</v>
       </c>
+      <c r="B32" t="s">
+        <v>1425</v>
+      </c>
       <c r="C32" t="s">
         <v>512</v>
       </c>
@@ -8855,6 +9175,9 @@
       <c r="A34" t="s">
         <v>515</v>
       </c>
+      <c r="B34" t="s">
+        <v>1426</v>
+      </c>
       <c r="C34" t="s">
         <v>516</v>
       </c>
@@ -8871,6 +9194,9 @@
       <c r="A36" t="s">
         <v>519</v>
       </c>
+      <c r="B36" t="s">
+        <v>1427</v>
+      </c>
       <c r="C36" t="s">
         <v>520</v>
       </c>
@@ -8887,6 +9213,9 @@
       <c r="A38" t="s">
         <v>523</v>
       </c>
+      <c r="B38" t="s">
+        <v>1428</v>
+      </c>
       <c r="C38" t="s">
         <v>524</v>
       </c>
@@ -8903,6 +9232,9 @@
       <c r="A40" t="s">
         <v>527</v>
       </c>
+      <c r="B40" t="s">
+        <v>1429</v>
+      </c>
       <c r="C40" t="s">
         <v>528</v>
       </c>
@@ -8919,6 +9251,9 @@
       <c r="A42" t="s">
         <v>531</v>
       </c>
+      <c r="B42" t="s">
+        <v>1430</v>
+      </c>
       <c r="C42" t="s">
         <v>532</v>
       </c>
@@ -8935,6 +9270,9 @@
       <c r="A44" t="s">
         <v>535</v>
       </c>
+      <c r="B44" t="s">
+        <v>1431</v>
+      </c>
       <c r="C44" t="s">
         <v>536</v>
       </c>
@@ -8951,6 +9289,9 @@
       <c r="A46" t="s">
         <v>539</v>
       </c>
+      <c r="B46" t="s">
+        <v>1432</v>
+      </c>
       <c r="C46" t="s">
         <v>540</v>
       </c>
@@ -8967,6 +9308,9 @@
       <c r="A48" t="s">
         <v>543</v>
       </c>
+      <c r="B48" t="s">
+        <v>1433</v>
+      </c>
       <c r="C48" t="s">
         <v>544</v>
       </c>
@@ -8983,6 +9327,9 @@
       <c r="A50" t="s">
         <v>547</v>
       </c>
+      <c r="B50" t="s">
+        <v>1434</v>
+      </c>
       <c r="C50" t="s">
         <v>548</v>
       </c>
@@ -8999,6 +9346,9 @@
       <c r="A52" t="s">
         <v>551</v>
       </c>
+      <c r="B52" t="s">
+        <v>1435</v>
+      </c>
       <c r="C52" t="s">
         <v>552</v>
       </c>
@@ -9015,6 +9365,9 @@
       <c r="A54" t="s">
         <v>555</v>
       </c>
+      <c r="B54" t="s">
+        <v>1436</v>
+      </c>
       <c r="C54" t="s">
         <v>556</v>
       </c>
@@ -9031,6 +9384,9 @@
       <c r="A56" t="s">
         <v>559</v>
       </c>
+      <c r="B56" t="s">
+        <v>1437</v>
+      </c>
       <c r="C56" t="s">
         <v>560</v>
       </c>
@@ -9047,6 +9403,9 @@
       <c r="A58" t="s">
         <v>563</v>
       </c>
+      <c r="B58" t="s">
+        <v>1438</v>
+      </c>
       <c r="C58" t="s">
         <v>564</v>
       </c>
@@ -9063,6 +9422,9 @@
       <c r="A60" t="s">
         <v>567</v>
       </c>
+      <c r="B60" t="s">
+        <v>1439</v>
+      </c>
       <c r="C60" t="s">
         <v>568</v>
       </c>
@@ -9079,6 +9441,9 @@
       <c r="A62" t="s">
         <v>571</v>
       </c>
+      <c r="B62" t="s">
+        <v>1440</v>
+      </c>
       <c r="C62" t="s">
         <v>572</v>
       </c>
@@ -9095,6 +9460,9 @@
       <c r="A64" t="s">
         <v>575</v>
       </c>
+      <c r="B64" t="s">
+        <v>1441</v>
+      </c>
       <c r="C64" t="s">
         <v>576</v>
       </c>
@@ -9111,6 +9479,9 @@
       <c r="A66" t="s">
         <v>579</v>
       </c>
+      <c r="B66" t="s">
+        <v>1442</v>
+      </c>
       <c r="C66" t="s">
         <v>580</v>
       </c>
@@ -9127,6 +9498,9 @@
       <c r="A68" t="s">
         <v>583</v>
       </c>
+      <c r="B68" t="s">
+        <v>1410</v>
+      </c>
       <c r="C68" t="s">
         <v>453</v>
       </c>
@@ -9143,6 +9517,9 @@
       <c r="A70" t="s">
         <v>585</v>
       </c>
+      <c r="B70" t="s">
+        <v>1443</v>
+      </c>
       <c r="C70" t="s">
         <v>586</v>
       </c>
@@ -9159,6 +9536,9 @@
       <c r="A72" t="s">
         <v>589</v>
       </c>
+      <c r="B72" t="s">
+        <v>1412</v>
+      </c>
       <c r="C72" t="s">
         <v>465</v>
       </c>
@@ -9175,6 +9555,9 @@
       <c r="A74" t="s">
         <v>591</v>
       </c>
+      <c r="B74" t="s">
+        <v>1444</v>
+      </c>
       <c r="C74" t="s">
         <v>592</v>
       </c>
@@ -9191,6 +9574,9 @@
       <c r="A76" t="s">
         <v>595</v>
       </c>
+      <c r="B76" t="s">
+        <v>1445</v>
+      </c>
       <c r="C76" t="s">
         <v>596</v>
       </c>
@@ -9207,6 +9593,9 @@
       <c r="A78" t="s">
         <v>599</v>
       </c>
+      <c r="B78" t="s">
+        <v>1446</v>
+      </c>
       <c r="C78" t="s">
         <v>600</v>
       </c>
@@ -9223,6 +9612,9 @@
       <c r="A80" t="s">
         <v>603</v>
       </c>
+      <c r="B80" t="s">
+        <v>1447</v>
+      </c>
       <c r="C80" t="s">
         <v>604</v>
       </c>
@@ -9239,6 +9631,9 @@
       <c r="A82" t="s">
         <v>607</v>
       </c>
+      <c r="B82" t="s">
+        <v>1416</v>
+      </c>
       <c r="C82" t="s">
         <v>481</v>
       </c>
@@ -9255,6 +9650,9 @@
       <c r="A84" t="s">
         <v>609</v>
       </c>
+      <c r="B84" t="s">
+        <v>1448</v>
+      </c>
       <c r="C84" t="s">
         <v>610</v>
       </c>
@@ -9271,6 +9669,9 @@
       <c r="A86" t="s">
         <v>613</v>
       </c>
+      <c r="B86" t="s">
+        <v>1449</v>
+      </c>
       <c r="C86" t="s">
         <v>614</v>
       </c>
@@ -9287,6 +9688,9 @@
       <c r="A88" t="s">
         <v>617</v>
       </c>
+      <c r="B88" t="s">
+        <v>1450</v>
+      </c>
       <c r="C88" t="s">
         <v>618</v>
       </c>
@@ -9303,6 +9707,9 @@
       <c r="A90" t="s">
         <v>621</v>
       </c>
+      <c r="B90" t="s">
+        <v>1451</v>
+      </c>
       <c r="C90" t="s">
         <v>622</v>
       </c>
@@ -9319,6 +9726,9 @@
       <c r="A92" t="s">
         <v>625</v>
       </c>
+      <c r="B92" t="s">
+        <v>1452</v>
+      </c>
       <c r="C92" t="s">
         <v>626</v>
       </c>
@@ -9335,6 +9745,9 @@
       <c r="A94" t="s">
         <v>629</v>
       </c>
+      <c r="B94" t="s">
+        <v>1453</v>
+      </c>
       <c r="C94" t="s">
         <v>630</v>
       </c>
@@ -9351,6 +9764,9 @@
       <c r="A96" t="s">
         <v>633</v>
       </c>
+      <c r="B96" t="s">
+        <v>1454</v>
+      </c>
       <c r="C96" t="s">
         <v>634</v>
       </c>
@@ -9367,6 +9783,9 @@
       <c r="A98" t="s">
         <v>637</v>
       </c>
+      <c r="B98" t="s">
+        <v>1455</v>
+      </c>
       <c r="C98" t="s">
         <v>638</v>
       </c>
@@ -9383,6 +9802,9 @@
       <c r="A100" t="s">
         <v>641</v>
       </c>
+      <c r="B100" t="s">
+        <v>1456</v>
+      </c>
       <c r="C100" t="s">
         <v>642</v>
       </c>
@@ -9399,6 +9821,9 @@
       <c r="A102" t="s">
         <v>645</v>
       </c>
+      <c r="B102" t="s">
+        <v>1457</v>
+      </c>
       <c r="C102" t="s">
         <v>646</v>
       </c>
@@ -9415,6 +9840,9 @@
       <c r="A104" t="s">
         <v>649</v>
       </c>
+      <c r="B104" t="s">
+        <v>1458</v>
+      </c>
       <c r="C104" t="s">
         <v>650</v>
       </c>
@@ -9431,6 +9859,9 @@
       <c r="A106" t="s">
         <v>653</v>
       </c>
+      <c r="B106" t="s">
+        <v>1459</v>
+      </c>
       <c r="C106" t="s">
         <v>654</v>
       </c>
@@ -9447,6 +9878,9 @@
       <c r="A108" t="s">
         <v>657</v>
       </c>
+      <c r="B108" t="s">
+        <v>1460</v>
+      </c>
       <c r="C108" t="s">
         <v>658</v>
       </c>
@@ -9463,6 +9897,9 @@
       <c r="A110" t="s">
         <v>661</v>
       </c>
+      <c r="B110" t="s">
+        <v>1461</v>
+      </c>
       <c r="C110" t="s">
         <v>662</v>
       </c>
@@ -9479,6 +9916,9 @@
       <c r="A112" t="s">
         <v>665</v>
       </c>
+      <c r="B112" t="s">
+        <v>1462</v>
+      </c>
       <c r="C112" t="s">
         <v>666</v>
       </c>
@@ -9495,6 +9935,9 @@
       <c r="A114" t="s">
         <v>669</v>
       </c>
+      <c r="B114" t="s">
+        <v>1463</v>
+      </c>
       <c r="C114" t="s">
         <v>670</v>
       </c>
@@ -9511,6 +9954,9 @@
       <c r="A116" t="s">
         <v>673</v>
       </c>
+      <c r="B116" t="s">
+        <v>1464</v>
+      </c>
       <c r="C116" t="s">
         <v>674</v>
       </c>
@@ -9527,6 +9973,9 @@
       <c r="A118" t="s">
         <v>677</v>
       </c>
+      <c r="B118" t="s">
+        <v>1465</v>
+      </c>
       <c r="C118" t="s">
         <v>678</v>
       </c>
@@ -9543,6 +9992,9 @@
       <c r="A120" t="s">
         <v>681</v>
       </c>
+      <c r="B120" t="s">
+        <v>1466</v>
+      </c>
       <c r="C120" t="s">
         <v>682</v>
       </c>
@@ -9559,6 +10011,9 @@
       <c r="A122" t="s">
         <v>685</v>
       </c>
+      <c r="B122" t="s">
+        <v>1467</v>
+      </c>
       <c r="C122" t="s">
         <v>686</v>
       </c>
@@ -9575,6 +10030,9 @@
       <c r="A124" t="s">
         <v>689</v>
       </c>
+      <c r="B124" t="s">
+        <v>1468</v>
+      </c>
       <c r="C124" t="s">
         <v>690</v>
       </c>
@@ -9591,6 +10049,9 @@
       <c r="A126" t="s">
         <v>693</v>
       </c>
+      <c r="B126" t="s">
+        <v>1469</v>
+      </c>
       <c r="C126" t="s">
         <v>694</v>
       </c>
@@ -9607,6 +10068,9 @@
       <c r="A128" t="s">
         <v>697</v>
       </c>
+      <c r="B128" t="s">
+        <v>1470</v>
+      </c>
       <c r="C128" t="s">
         <v>698</v>
       </c>
@@ -9623,6 +10087,9 @@
       <c r="A130" t="s">
         <v>701</v>
       </c>
+      <c r="B130" t="s">
+        <v>1471</v>
+      </c>
       <c r="C130" t="s">
         <v>702</v>
       </c>
@@ -9639,6 +10106,9 @@
       <c r="A132" t="s">
         <v>705</v>
       </c>
+      <c r="B132" t="s">
+        <v>1472</v>
+      </c>
       <c r="C132" t="s">
         <v>706</v>
       </c>
@@ -9655,6 +10125,9 @@
       <c r="A134" t="s">
         <v>709</v>
       </c>
+      <c r="B134" t="s">
+        <v>1473</v>
+      </c>
       <c r="C134" t="s">
         <v>710</v>
       </c>
@@ -9671,6 +10144,9 @@
       <c r="A136" t="s">
         <v>713</v>
       </c>
+      <c r="B136" t="s">
+        <v>1474</v>
+      </c>
       <c r="C136" t="s">
         <v>714</v>
       </c>
@@ -9687,6 +10163,9 @@
       <c r="A138" t="s">
         <v>717</v>
       </c>
+      <c r="B138" t="s">
+        <v>1475</v>
+      </c>
       <c r="C138" t="s">
         <v>718</v>
       </c>
@@ -9703,6 +10182,9 @@
       <c r="A140" t="s">
         <v>721</v>
       </c>
+      <c r="B140" t="s">
+        <v>1476</v>
+      </c>
       <c r="C140" t="s">
         <v>722</v>
       </c>
@@ -9719,6 +10201,9 @@
       <c r="A142" t="s">
         <v>725</v>
       </c>
+      <c r="B142" t="s">
+        <v>1477</v>
+      </c>
       <c r="C142" t="s">
         <v>726</v>
       </c>
@@ -9735,6 +10220,9 @@
       <c r="A144" t="s">
         <v>729</v>
       </c>
+      <c r="B144" t="s">
+        <v>1478</v>
+      </c>
       <c r="C144" t="s">
         <v>730</v>
       </c>
@@ -9751,6 +10239,9 @@
       <c r="A146" t="s">
         <v>733</v>
       </c>
+      <c r="B146" t="s">
+        <v>1479</v>
+      </c>
       <c r="C146" t="s">
         <v>734</v>
       </c>
@@ -9767,6 +10258,9 @@
       <c r="A148" t="s">
         <v>737</v>
       </c>
+      <c r="B148" t="s">
+        <v>1480</v>
+      </c>
       <c r="C148" t="s">
         <v>738</v>
       </c>
@@ -9783,6 +10277,9 @@
       <c r="A150" t="s">
         <v>741</v>
       </c>
+      <c r="B150" t="s">
+        <v>1481</v>
+      </c>
       <c r="C150" t="s">
         <v>742</v>
       </c>
@@ -9799,6 +10296,9 @@
       <c r="A152" t="s">
         <v>745</v>
       </c>
+      <c r="B152" t="s">
+        <v>1482</v>
+      </c>
       <c r="C152" t="s">
         <v>746</v>
       </c>
@@ -9815,6 +10315,9 @@
       <c r="A154" t="s">
         <v>749</v>
       </c>
+      <c r="B154" t="s">
+        <v>1483</v>
+      </c>
       <c r="C154" t="s">
         <v>750</v>
       </c>
@@ -9831,6 +10334,9 @@
       <c r="A156" t="s">
         <v>753</v>
       </c>
+      <c r="B156" t="s">
+        <v>1484</v>
+      </c>
       <c r="C156" t="s">
         <v>754</v>
       </c>
@@ -9847,6 +10353,9 @@
       <c r="A158" t="s">
         <v>757</v>
       </c>
+      <c r="B158" t="s">
+        <v>1485</v>
+      </c>
       <c r="C158" t="s">
         <v>758</v>
       </c>
@@ -9863,6 +10372,9 @@
       <c r="A160" t="s">
         <v>761</v>
       </c>
+      <c r="B160" t="s">
+        <v>1486</v>
+      </c>
       <c r="C160" t="s">
         <v>762</v>
       </c>
@@ -9879,6 +10391,9 @@
       <c r="A162" t="s">
         <v>765</v>
       </c>
+      <c r="B162" t="s">
+        <v>1487</v>
+      </c>
       <c r="C162" t="s">
         <v>766</v>
       </c>
@@ -9895,6 +10410,9 @@
       <c r="A164" t="s">
         <v>769</v>
       </c>
+      <c r="B164" t="s">
+        <v>1488</v>
+      </c>
       <c r="C164" t="s">
         <v>770</v>
       </c>
@@ -9911,6 +10429,9 @@
       <c r="A166" t="s">
         <v>773</v>
       </c>
+      <c r="B166" t="s">
+        <v>1489</v>
+      </c>
       <c r="C166" t="s">
         <v>774</v>
       </c>
@@ -9927,6 +10448,9 @@
       <c r="A168" t="s">
         <v>777</v>
       </c>
+      <c r="B168" t="s">
+        <v>1490</v>
+      </c>
       <c r="C168" t="s">
         <v>778</v>
       </c>
@@ -9943,6 +10467,9 @@
       <c r="A170" t="s">
         <v>781</v>
       </c>
+      <c r="B170" t="s">
+        <v>1491</v>
+      </c>
       <c r="C170" t="s">
         <v>782</v>
       </c>
@@ -9959,6 +10486,9 @@
       <c r="A172" t="s">
         <v>785</v>
       </c>
+      <c r="B172" t="s">
+        <v>1492</v>
+      </c>
       <c r="C172" t="s">
         <v>786</v>
       </c>
@@ -9974,6 +10504,9 @@
     <row r="174" spans="1:3">
       <c r="A174" t="s">
         <v>789</v>
+      </c>
+      <c r="B174" t="s">
+        <v>1493</v>
       </c>
       <c r="C174" t="s">
         <v>790</v>
@@ -10701,7 +11234,7 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="9" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>1155</v>
@@ -10712,7 +11245,7 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="9" t="s">
-        <v>1232</v>
+        <v>1230</v>
       </c>
       <c r="B37" s="9" t="s">
         <v>1156</v>
@@ -10723,7 +11256,7 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="9" t="s">
-        <v>1233</v>
+        <v>1231</v>
       </c>
       <c r="B38" s="9" t="s">
         <v>1157</v>
@@ -10734,7 +11267,7 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="9" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
       <c r="B39" s="9" t="s">
         <v>1153</v>
@@ -10745,7 +11278,7 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="9" t="s">
-        <v>1235</v>
+        <v>1233</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>1154</v>
@@ -10756,7 +11289,7 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="9" t="s">
-        <v>1236</v>
+        <v>1234</v>
       </c>
       <c r="B41" s="9" t="s">
         <v>1158</v>
@@ -10767,7 +11300,7 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="9" t="s">
-        <v>1237</v>
+        <v>1235</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>1159</v>
@@ -10778,7 +11311,7 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="9" t="s">
-        <v>1238</v>
+        <v>1236</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>1161</v>
@@ -10789,7 +11322,7 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="9" t="s">
-        <v>1239</v>
+        <v>1237</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>1160</v>
@@ -10800,7 +11333,7 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="9" t="s">
-        <v>1240</v>
+        <v>1238</v>
       </c>
       <c r="B45" s="9" t="s">
         <v>1162</v>
@@ -10811,7 +11344,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="9" t="s">
-        <v>1241</v>
+        <v>1239</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>1163</v>
@@ -10822,7 +11355,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="9" t="s">
-        <v>1242</v>
+        <v>1240</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>1164</v>
@@ -10833,7 +11366,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="9" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>1165</v>
@@ -10844,7 +11377,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="9" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
       <c r="B49" s="9" t="s">
         <v>1166</v>
@@ -10855,7 +11388,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="9" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>1167</v>
@@ -10866,7 +11399,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="9" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="B51" s="9" t="s">
         <v>1168</v>
@@ -10877,7 +11410,7 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="9" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>1169</v>
@@ -10888,7 +11421,7 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="9" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>1170</v>
@@ -10899,7 +11432,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="9" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="B54" s="9" t="s">
         <v>1171</v>
@@ -10910,7 +11443,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="9" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>1172</v>
@@ -10921,7 +11454,7 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="9" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="B56" s="9" t="s">
         <v>1173</v>
@@ -10932,7 +11465,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="9" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>1175</v>
@@ -10943,7 +11476,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="9" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="B58" s="9" t="s">
         <v>1174</v>
@@ -10954,7 +11487,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="9" t="s">
-        <v>1254</v>
+        <v>1252</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>1176</v>
@@ -10965,7 +11498,7 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="9" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="B60" s="9" t="s">
         <v>1177</v>

</xml_diff>

<commit_message>
Update for leaving messages
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -1,35 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\ProjectMT3SA\ProjectMT3\Data\Locale\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05565F7-69A6-401A-9814-1867478C7723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-32560" yWindow="2030" windowWidth="28800" windowHeight="15370" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="UI" sheetId="1" r:id="rId1"/>
-    <sheet name="Languages" sheetId="2" r:id="rId2"/>
-    <sheet name="Attrs" sheetId="3" r:id="rId3"/>
-    <sheet name="Items" sheetId="4" r:id="rId4"/>
-    <sheet name="Enemies" sheetId="5" r:id="rId5"/>
-    <sheet name="Equips" sheetId="6" r:id="rId6"/>
-    <sheet name="Classes" sheetId="7" r:id="rId7"/>
-    <sheet name="States" sheetId="8" r:id="rId8"/>
-    <sheet name="MapNames" sheetId="9" r:id="rId9"/>
-    <sheet name="Specials" sheetId="10" r:id="rId10"/>
-    <sheet name="Player" sheetId="11" r:id="rId11"/>
-    <sheet name="DialogueNames" sheetId="12" r:id="rId12"/>
-    <sheet name="DialogueContents" sheetId="13" r:id="rId13"/>
-    <sheet name="TutorialMessages" sheetId="15" r:id="rId14"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+  <ns0:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <ns0:workbookPr/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="D:\Dev\ProjectMT3SA\ProjectMT3\Data\Locale\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05565F7-69A6-401A-9814-1867478C7723}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns0:bookViews>
+    <ns0:workbookView xWindow="-32560" yWindow="2030" windowWidth="28800" windowHeight="15370" firstSheet="3" activeTab="8" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="UI" sheetId="1" ns7:id="rId1"/>
+    <ns0:sheet name="Languages" sheetId="2" ns7:id="rId2"/>
+    <ns0:sheet name="Attrs" sheetId="3" ns7:id="rId3"/>
+    <ns0:sheet name="Items" sheetId="4" ns7:id="rId4"/>
+    <ns0:sheet name="Enemies" sheetId="5" ns7:id="rId5"/>
+    <ns0:sheet name="Equips" sheetId="6" ns7:id="rId6"/>
+    <ns0:sheet name="Classes" sheetId="7" ns7:id="rId7"/>
+    <ns0:sheet name="States" sheetId="8" ns7:id="rId8"/>
+    <ns0:sheet name="MapNames" sheetId="9" ns7:id="rId9"/>
+    <ns0:sheet name="Specials" sheetId="10" ns7:id="rId10"/>
+    <ns0:sheet name="Player" sheetId="11" ns7:id="rId11"/>
+    <ns0:sheet name="DialogueNames" sheetId="12" ns7:id="rId12"/>
+    <ns0:sheet name="DialogueContents" sheetId="13" ns7:id="rId13"/>
+    <ns0:sheet name="TutorialMessages" sheetId="15" ns7:id="rId14"/>
+    <ns0:sheet name="messages" sheetId="15" ns7:id="rId18"/>
+  </ns0:sheets>
+  <ns0:calcPr calcId="0"/>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8181,6 +8182,394 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="37" hidden="0" customWidth="1"/>
+    <ns0:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <ns0:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="str" s="1">
+        <ns0:v>ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="str" s="1">
+        <ns0:v>en_GB</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="str" s="1">
+        <ns0:v>zh_CN</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_LABEL</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" t="str">
+        <ns0:v>Template</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" t="str">
+        <ns0:v>句式</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" t="str">
+        <ns0:v>MESSAGES_WORD_LABEL</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" t="str">
+        <ns0:v>Word</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" t="str">
+        <ns0:v>词语</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" t="str">
+        <ns0:v>MESSAGES_PUBLISH</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" t="str">
+        <ns0:v>Confirm</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" t="str">
+        <ns0:v>确认</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="str">
+        <ns0:v>MESSAGES_HOTKEY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" t="str">
+        <ns0:v>T: Leave a message</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" t="str">
+        <ns0:v>T：留下箴言</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="str">
+        <ns0:v>MESSAGES_NETWORK_BAD</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" t="str">
+        <ns0:v>Poor network connection. Please try again later.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" t="str">
+        <ns0:v>当前网络环境不佳，请稍后再试。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="str">
+        <ns0:v>MESSAGES_CHECKING</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" t="str">
+        <ns0:v>Checking connection…</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" t="str">
+        <ns0:v>正在检测网络连接……</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="str">
+        <ns0:v>MESSAGES_OFFLINE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B8" t="str">
+        <ns0:v>Connection unavailable</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" t="str">
+        <ns0:v>当前网络环境不佳</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="str">
+        <ns0:v>MESSAGES_READY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B9" t="str">
+        <ns0:v>Ready to publish</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" t="str">
+        <ns0:v>可以发布留言</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" t="str">
+        <ns0:v>MESSAGES_SENDING</ns0:v>
+      </ns0:c>
+      <ns0:c r="B10" t="str">
+        <ns0:v>Publishing…</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" t="str">
+        <ns0:v>正在发布……</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" t="str">
+        <ns0:v>MESSAGES_SENT</ns0:v>
+      </ns0:c>
+      <ns0:c r="B11" t="str">
+        <ns0:v>Message published.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" t="str">
+        <ns0:v>留言已发布。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" t="str">
+        <ns0:v>MESSAGES_FAILED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B12" t="str">
+        <ns0:v>Could not publish. The local message was removed.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C12" t="str">
+        <ns0:v>留言发布失败，已移除本地留言。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" t="str">
+        <ns0:v>MESSAGES_RATE_LIMITED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B13" t="str">
+        <ns0:v>Please wait {seconds} seconds before publishing again.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C13" t="str">
+        <ns0:v>请等待 {seconds} 秒后再发布留言。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_AHEAD</ns0:v>
+      </ns0:c>
+      <ns0:c r="B14" t="str">
+        <ns0:v>{word} ahead</ns0:v>
+      </ns0:c>
+      <ns0:c r="C14" t="str">
+        <ns0:v>前方有{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_BEWARE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B15" t="str">
+        <ns0:v>Beware of {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C15" t="str">
+        <ns0:v>小心{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_SEEK</ns0:v>
+      </ns0:c>
+      <ns0:c r="B16" t="str">
+        <ns0:v>Seek {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C16" t="str">
+        <ns0:v>寻找{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_REMEMBER</ns0:v>
+      </ns0:c>
+      <ns0:c r="B17" t="str">
+        <ns0:v>Do not forget {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C17" t="str">
+        <ns0:v>别忘了{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_NEED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B18" t="str">
+        <ns0:v>{word} required</ns0:v>
+      </ns0:c>
+      <ns0:c r="C18" t="str">
+        <ns0:v>需要{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" t="str">
+        <ns0:v>MESSAGES_WORD_ENEMY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B19" t="str">
+        <ns0:v>a strong enemy</ns0:v>
+      </ns0:c>
+      <ns0:c r="C19" t="str">
+        <ns0:v>强敌</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" t="str">
+        <ns0:v>MESSAGES_WORD_AMBUSH</ns0:v>
+      </ns0:c>
+      <ns0:c r="B20" t="str">
+        <ns0:v>an ambush</ns0:v>
+      </ns0:c>
+      <ns0:c r="C20" t="str">
+        <ns0:v>伏击</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" t="str">
+        <ns0:v>MESSAGES_WORD_TRAP</ns0:v>
+      </ns0:c>
+      <ns0:c r="B21" t="str">
+        <ns0:v>a trap</ns0:v>
+      </ns0:c>
+      <ns0:c r="C21" t="str">
+        <ns0:v>陷阱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" t="str">
+        <ns0:v>MESSAGES_WORD_POISON</ns0:v>
+      </ns0:c>
+      <ns0:c r="B22" t="str">
+        <ns0:v>poison</ns0:v>
+      </ns0:c>
+      <ns0:c r="C22" t="str">
+        <ns0:v>中毒</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" t="str">
+        <ns0:v>MESSAGES_WORD_WEAKNESS</ns0:v>
+      </ns0:c>
+      <ns0:c r="B23" t="str">
+        <ns0:v>weakness</ns0:v>
+      </ns0:c>
+      <ns0:c r="C23" t="str">
+        <ns0:v>衰弱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" t="str">
+        <ns0:v>MESSAGES_WORD_MECHANISM</ns0:v>
+      </ns0:c>
+      <ns0:c r="B24" t="str">
+        <ns0:v>a mechanism</ns0:v>
+      </ns0:c>
+      <ns0:c r="C24" t="str">
+        <ns0:v>机关</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" t="str">
+        <ns0:v>MESSAGES_WORD_PASSAGE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B25" t="str">
+        <ns0:v>a hidden passage</ns0:v>
+      </ns0:c>
+      <ns0:c r="C25" t="str">
+        <ns0:v>暗道</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" t="str">
+        <ns0:v>MESSAGES_WORD_STAIRS</ns0:v>
+      </ns0:c>
+      <ns0:c r="B26" t="str">
+        <ns0:v>stairs</ns0:v>
+      </ns0:c>
+      <ns0:c r="C26" t="str">
+        <ns0:v>楼梯</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" t="str">
+        <ns0:v>MESSAGES_WORD_KEY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" t="str">
+        <ns0:v>a key</ns0:v>
+      </ns0:c>
+      <ns0:c r="C27" t="str">
+        <ns0:v>钥匙</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" t="str">
+        <ns0:v>MESSAGES_WORD_POTION</ns0:v>
+      </ns0:c>
+      <ns0:c r="B28" t="str">
+        <ns0:v>a potion</ns0:v>
+      </ns0:c>
+      <ns0:c r="C28" t="str">
+        <ns0:v>药水</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" t="str">
+        <ns0:v>MESSAGES_WORD_GEM</ns0:v>
+      </ns0:c>
+      <ns0:c r="B29" t="str">
+        <ns0:v>a gem</ns0:v>
+      </ns0:c>
+      <ns0:c r="C29" t="str">
+        <ns0:v>宝石</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" t="str">
+        <ns0:v>MESSAGES_WORD_CHEST</ns0:v>
+      </ns0:c>
+      <ns0:c r="B30" t="str">
+        <ns0:v>a chest</ns0:v>
+      </ns0:c>
+      <ns0:c r="C30" t="str">
+        <ns0:v>宝箱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" t="str">
+        <ns0:v>MESSAGES_WORD_SHOP</ns0:v>
+      </ns0:c>
+      <ns0:c r="B31" t="str">
+        <ns0:v>a shop</ns0:v>
+      </ns0:c>
+      <ns0:c r="C31" t="str">
+        <ns0:v>商店</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" t="str">
+        <ns0:v>MESSAGES_WORD_WEAPON</ns0:v>
+      </ns0:c>
+      <ns0:c r="B32" t="str">
+        <ns0:v>a weapon</ns0:v>
+      </ns0:c>
+      <ns0:c r="C32" t="str">
+        <ns0:v>武器</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" t="str">
+        <ns0:v>MESSAGES_WORD_ARMOUR</ns0:v>
+      </ns0:c>
+      <ns0:c r="B33" t="str">
+        <ns0:v>armour</ns0:v>
+      </ns0:c>
+      <ns0:c r="C33" t="str">
+        <ns0:v>防具</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34">
+      <ns0:c r="A34" t="str">
+        <ns0:v>MESSAGES_WORD_TELEPORTER</ns0:v>
+      </ns0:c>
+      <ns0:c r="B34" t="str">
+        <ns0:v>a teleporter</ns0:v>
+      </ns0:c>
+      <ns0:c r="C34" t="str">
+        <ns0:v>传送点</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>

</xml_diff>

<commit_message>
chore: sync Ludork Engine, Global, Internal, Enums and Lua stubs (#32)
* chore: sync Ludork Engine, Global, Internal, Enums and Lua stubs from 08bd83caf61b0ac4bc64baac1ecde709433a72e5

* Update CI

* Add basic metas

* Update for leaving messages

---------

Co-authored-by: JasonLeon01 <118749439+JasonLeon01@users.noreply.github.com>
Co-authored-by: Jason Leon <jasonleon01@outlook.com>
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -1,35 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\ProjectMT3SA\ProjectMT3\Data\Locale\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05565F7-69A6-401A-9814-1867478C7723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-32560" yWindow="2030" windowWidth="28800" windowHeight="15370" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="UI" sheetId="1" r:id="rId1"/>
-    <sheet name="Languages" sheetId="2" r:id="rId2"/>
-    <sheet name="Attrs" sheetId="3" r:id="rId3"/>
-    <sheet name="Items" sheetId="4" r:id="rId4"/>
-    <sheet name="Enemies" sheetId="5" r:id="rId5"/>
-    <sheet name="Equips" sheetId="6" r:id="rId6"/>
-    <sheet name="Classes" sheetId="7" r:id="rId7"/>
-    <sheet name="States" sheetId="8" r:id="rId8"/>
-    <sheet name="MapNames" sheetId="9" r:id="rId9"/>
-    <sheet name="Specials" sheetId="10" r:id="rId10"/>
-    <sheet name="Player" sheetId="11" r:id="rId11"/>
-    <sheet name="DialogueNames" sheetId="12" r:id="rId12"/>
-    <sheet name="DialogueContents" sheetId="13" r:id="rId13"/>
-    <sheet name="TutorialMessages" sheetId="15" r:id="rId14"/>
-  </sheets>
-  <calcPr calcId="0"/>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+  <ns0:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <ns0:workbookPr/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="D:\Dev\ProjectMT3SA\ProjectMT3\Data\Locale\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05565F7-69A6-401A-9814-1867478C7723}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns0:bookViews>
+    <ns0:workbookView xWindow="-32560" yWindow="2030" windowWidth="28800" windowHeight="15370" firstSheet="3" activeTab="8" ns6:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="UI" sheetId="1" ns7:id="rId1"/>
+    <ns0:sheet name="Languages" sheetId="2" ns7:id="rId2"/>
+    <ns0:sheet name="Attrs" sheetId="3" ns7:id="rId3"/>
+    <ns0:sheet name="Items" sheetId="4" ns7:id="rId4"/>
+    <ns0:sheet name="Enemies" sheetId="5" ns7:id="rId5"/>
+    <ns0:sheet name="Equips" sheetId="6" ns7:id="rId6"/>
+    <ns0:sheet name="Classes" sheetId="7" ns7:id="rId7"/>
+    <ns0:sheet name="States" sheetId="8" ns7:id="rId8"/>
+    <ns0:sheet name="MapNames" sheetId="9" ns7:id="rId9"/>
+    <ns0:sheet name="Specials" sheetId="10" ns7:id="rId10"/>
+    <ns0:sheet name="Player" sheetId="11" ns7:id="rId11"/>
+    <ns0:sheet name="DialogueNames" sheetId="12" ns7:id="rId12"/>
+    <ns0:sheet name="DialogueContents" sheetId="13" ns7:id="rId13"/>
+    <ns0:sheet name="TutorialMessages" sheetId="15" ns7:id="rId14"/>
+    <ns0:sheet name="messages" sheetId="15" ns7:id="rId18"/>
+  </ns0:sheets>
+  <ns0:calcPr calcId="0"/>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8181,6 +8182,394 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="37" hidden="0" customWidth="1"/>
+    <ns0:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <ns0:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="str" s="1">
+        <ns0:v>ID</ns0:v>
+      </ns0:c>
+      <ns0:c r="B1" t="str" s="1">
+        <ns0:v>en_GB</ns0:v>
+      </ns0:c>
+      <ns0:c r="C1" t="str" s="1">
+        <ns0:v>zh_CN</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_LABEL</ns0:v>
+      </ns0:c>
+      <ns0:c r="B2" t="str">
+        <ns0:v>Template</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" t="str">
+        <ns0:v>句式</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" t="str">
+        <ns0:v>MESSAGES_WORD_LABEL</ns0:v>
+      </ns0:c>
+      <ns0:c r="B3" t="str">
+        <ns0:v>Word</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" t="str">
+        <ns0:v>词语</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" t="str">
+        <ns0:v>MESSAGES_PUBLISH</ns0:v>
+      </ns0:c>
+      <ns0:c r="B4" t="str">
+        <ns0:v>Confirm</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" t="str">
+        <ns0:v>确认</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" t="str">
+        <ns0:v>MESSAGES_HOTKEY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" t="str">
+        <ns0:v>T: Leave a message</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" t="str">
+        <ns0:v>T：留下箴言</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" t="str">
+        <ns0:v>MESSAGES_NETWORK_BAD</ns0:v>
+      </ns0:c>
+      <ns0:c r="B6" t="str">
+        <ns0:v>Poor network connection. Please try again later.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" t="str">
+        <ns0:v>当前网络环境不佳，请稍后再试。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" t="str">
+        <ns0:v>MESSAGES_CHECKING</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" t="str">
+        <ns0:v>Checking connection…</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" t="str">
+        <ns0:v>正在检测网络连接……</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" t="str">
+        <ns0:v>MESSAGES_OFFLINE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B8" t="str">
+        <ns0:v>Connection unavailable</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" t="str">
+        <ns0:v>当前网络环境不佳</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" t="str">
+        <ns0:v>MESSAGES_READY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B9" t="str">
+        <ns0:v>Ready to publish</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" t="str">
+        <ns0:v>可以发布留言</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" t="str">
+        <ns0:v>MESSAGES_SENDING</ns0:v>
+      </ns0:c>
+      <ns0:c r="B10" t="str">
+        <ns0:v>Publishing…</ns0:v>
+      </ns0:c>
+      <ns0:c r="C10" t="str">
+        <ns0:v>正在发布……</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" t="str">
+        <ns0:v>MESSAGES_SENT</ns0:v>
+      </ns0:c>
+      <ns0:c r="B11" t="str">
+        <ns0:v>Message published.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C11" t="str">
+        <ns0:v>留言已发布。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" t="str">
+        <ns0:v>MESSAGES_FAILED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B12" t="str">
+        <ns0:v>Could not publish. The local message was removed.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C12" t="str">
+        <ns0:v>留言发布失败，已移除本地留言。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" t="str">
+        <ns0:v>MESSAGES_RATE_LIMITED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B13" t="str">
+        <ns0:v>Please wait {seconds} seconds before publishing again.</ns0:v>
+      </ns0:c>
+      <ns0:c r="C13" t="str">
+        <ns0:v>请等待 {seconds} 秒后再发布留言。</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_AHEAD</ns0:v>
+      </ns0:c>
+      <ns0:c r="B14" t="str">
+        <ns0:v>{word} ahead</ns0:v>
+      </ns0:c>
+      <ns0:c r="C14" t="str">
+        <ns0:v>前方有{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_BEWARE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B15" t="str">
+        <ns0:v>Beware of {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C15" t="str">
+        <ns0:v>小心{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_SEEK</ns0:v>
+      </ns0:c>
+      <ns0:c r="B16" t="str">
+        <ns0:v>Seek {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C16" t="str">
+        <ns0:v>寻找{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_REMEMBER</ns0:v>
+      </ns0:c>
+      <ns0:c r="B17" t="str">
+        <ns0:v>Do not forget {word}</ns0:v>
+      </ns0:c>
+      <ns0:c r="C17" t="str">
+        <ns0:v>别忘了{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" t="str">
+        <ns0:v>MESSAGES_TEMPLATE_NEED</ns0:v>
+      </ns0:c>
+      <ns0:c r="B18" t="str">
+        <ns0:v>{word} required</ns0:v>
+      </ns0:c>
+      <ns0:c r="C18" t="str">
+        <ns0:v>需要{word}</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" t="str">
+        <ns0:v>MESSAGES_WORD_ENEMY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B19" t="str">
+        <ns0:v>a strong enemy</ns0:v>
+      </ns0:c>
+      <ns0:c r="C19" t="str">
+        <ns0:v>强敌</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" t="str">
+        <ns0:v>MESSAGES_WORD_AMBUSH</ns0:v>
+      </ns0:c>
+      <ns0:c r="B20" t="str">
+        <ns0:v>an ambush</ns0:v>
+      </ns0:c>
+      <ns0:c r="C20" t="str">
+        <ns0:v>伏击</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" t="str">
+        <ns0:v>MESSAGES_WORD_TRAP</ns0:v>
+      </ns0:c>
+      <ns0:c r="B21" t="str">
+        <ns0:v>a trap</ns0:v>
+      </ns0:c>
+      <ns0:c r="C21" t="str">
+        <ns0:v>陷阱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" t="str">
+        <ns0:v>MESSAGES_WORD_POISON</ns0:v>
+      </ns0:c>
+      <ns0:c r="B22" t="str">
+        <ns0:v>poison</ns0:v>
+      </ns0:c>
+      <ns0:c r="C22" t="str">
+        <ns0:v>中毒</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" t="str">
+        <ns0:v>MESSAGES_WORD_WEAKNESS</ns0:v>
+      </ns0:c>
+      <ns0:c r="B23" t="str">
+        <ns0:v>weakness</ns0:v>
+      </ns0:c>
+      <ns0:c r="C23" t="str">
+        <ns0:v>衰弱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" t="str">
+        <ns0:v>MESSAGES_WORD_MECHANISM</ns0:v>
+      </ns0:c>
+      <ns0:c r="B24" t="str">
+        <ns0:v>a mechanism</ns0:v>
+      </ns0:c>
+      <ns0:c r="C24" t="str">
+        <ns0:v>机关</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" t="str">
+        <ns0:v>MESSAGES_WORD_PASSAGE</ns0:v>
+      </ns0:c>
+      <ns0:c r="B25" t="str">
+        <ns0:v>a hidden passage</ns0:v>
+      </ns0:c>
+      <ns0:c r="C25" t="str">
+        <ns0:v>暗道</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" t="str">
+        <ns0:v>MESSAGES_WORD_STAIRS</ns0:v>
+      </ns0:c>
+      <ns0:c r="B26" t="str">
+        <ns0:v>stairs</ns0:v>
+      </ns0:c>
+      <ns0:c r="C26" t="str">
+        <ns0:v>楼梯</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" t="str">
+        <ns0:v>MESSAGES_WORD_KEY</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" t="str">
+        <ns0:v>a key</ns0:v>
+      </ns0:c>
+      <ns0:c r="C27" t="str">
+        <ns0:v>钥匙</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" t="str">
+        <ns0:v>MESSAGES_WORD_POTION</ns0:v>
+      </ns0:c>
+      <ns0:c r="B28" t="str">
+        <ns0:v>a potion</ns0:v>
+      </ns0:c>
+      <ns0:c r="C28" t="str">
+        <ns0:v>药水</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" t="str">
+        <ns0:v>MESSAGES_WORD_GEM</ns0:v>
+      </ns0:c>
+      <ns0:c r="B29" t="str">
+        <ns0:v>a gem</ns0:v>
+      </ns0:c>
+      <ns0:c r="C29" t="str">
+        <ns0:v>宝石</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" t="str">
+        <ns0:v>MESSAGES_WORD_CHEST</ns0:v>
+      </ns0:c>
+      <ns0:c r="B30" t="str">
+        <ns0:v>a chest</ns0:v>
+      </ns0:c>
+      <ns0:c r="C30" t="str">
+        <ns0:v>宝箱</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" t="str">
+        <ns0:v>MESSAGES_WORD_SHOP</ns0:v>
+      </ns0:c>
+      <ns0:c r="B31" t="str">
+        <ns0:v>a shop</ns0:v>
+      </ns0:c>
+      <ns0:c r="C31" t="str">
+        <ns0:v>商店</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" t="str">
+        <ns0:v>MESSAGES_WORD_WEAPON</ns0:v>
+      </ns0:c>
+      <ns0:c r="B32" t="str">
+        <ns0:v>a weapon</ns0:v>
+      </ns0:c>
+      <ns0:c r="C32" t="str">
+        <ns0:v>武器</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" t="str">
+        <ns0:v>MESSAGES_WORD_ARMOUR</ns0:v>
+      </ns0:c>
+      <ns0:c r="B33" t="str">
+        <ns0:v>armour</ns0:v>
+      </ns0:c>
+      <ns0:c r="C33" t="str">
+        <ns0:v>防具</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34">
+      <ns0:c r="A34" t="str">
+        <ns0:v>MESSAGES_WORD_TELEPORTER</ns0:v>
+      </ns0:c>
+      <ns0:c r="B34" t="str">
+        <ns0:v>a teleporter</ns0:v>
+      </ns0:c>
+      <ns0:c r="C34" t="str">
+        <ns0:v>传送点</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</ns0:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C3"/>

</xml_diff>

<commit_message>
Update control for multi-platforms
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -5025,7 +5025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -5705,14 +5705,20 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>259</v>
-      </c>
-      <c r="B62" t="s">
-        <v>260</v>
-      </c>
-      <c r="C62" t="s">
-        <v>261</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BATTLE_RETREAT</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Retreat</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>撤退</t>
+        </is>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -5867,6 +5873,210 @@
       </c>
       <c r="C76" t="s">
         <v>1300</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CONTROLS_TITLE</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>HOTKEY_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>H: Controls</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>H：操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>HOTKEY_BATTLE</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Battle — Q: Retreat; C: Critical hit; Z/X: Attack/defense skill</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>战斗：Q 撤退，C 会心一击，Z/X 攻击/防御技能</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>GAMEPAD_MOVE</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Left stick / D-pad: Move</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>左摇杆／十字键：移动</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>GAMEPAD_MENU</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Menu: Open menu</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>菜单键：打开菜单</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>GAMEPAD_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>X: Controls</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>X：操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>GAMEPAD_CONFIRM</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>A: Confirm; B: Back</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>A：确认；B：返回</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>GAMEPAD_BATTLE</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Battle — B: Retreat; A: Critical hit; D-pad left/right: Attack/defense skill</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>战斗：B 撤退，A 会心一击，十字键左/右使用攻击/防御技能</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>TOUCH_MOVE</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Tap the map: Move to the destination</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>点击地图：移动到目标位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>TOUCH_MENU</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Tap an avatar: Menu; swipe avatars: Switch party member</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>点击头像：菜单；左右滑动头像：切换角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TOUCH_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Tap Controls to view the controls</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>点击操作说明查看操作方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TOUCH_BATTLE</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Battle: Tap the skill, critical hit or retreat button</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>战斗：点击技能、会心一击或撤退按钮</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8059,7 +8269,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4933D5-C722-C646-96A3-51CA5B4C6607}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="43" customWidth="1"/>
@@ -8111,14 +8321,20 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>1199</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1265</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>1266</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TM_04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Press H to view the controls.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>按 H 键可以查看操作说明。</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -8174,6 +8390,74 @@
       </c>
       <c r="C10" s="2" t="s">
         <v>1458</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TM_04_G</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Press X to view the controls.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>按 X 键可以查看操作说明。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TM_04_M</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tap Controls to view the controls.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>点击操作说明可以查看操作方式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TM_05_G</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Enemy information. Press A to view details.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>敌人的能力信息，按 A 查看详细内容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TM_07_MENU</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Open Items from the menu to use this item.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>打开菜单中的道具来使用。</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8565,6 +8849,40 @@
         <ns0:v>传送点</ns0:v>
       </ns0:c>
     </ns0:row>
+    <ns0:row r="35">
+      <ns0:c r="A35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MESSAGES_GAMEPAD_HOTKEY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Y: Leave a message</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Y：留言</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36">
+      <ns0:c r="A36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MESSAGES_TOUCH_HOTKEY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hold your current tile: Leave a message</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>长按角色当前格子：留言</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
   </ns0:sheetData>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </ns0:worksheet>

</xml_diff>

<commit_message>
chore: sync Ludork Engine, Global, Internal, Enums and Lua stubs (#33)
* chore: sync Ludork Engine, Global, Internal, Enums and Lua stubs from cf17416f170d2cabb056473bfe71169052271b1e

* Update control for multi-platforms

---------

Co-authored-by: JasonLeon01 <118749439+JasonLeon01@users.noreply.github.com>
Co-authored-by: Jason Leon <jasonleon01@outlook.com>
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -5025,7 +5025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -5705,14 +5705,20 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>259</v>
-      </c>
-      <c r="B62" t="s">
-        <v>260</v>
-      </c>
-      <c r="C62" t="s">
-        <v>261</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BATTLE_RETREAT</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Retreat</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>撤退</t>
+        </is>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -5867,6 +5873,210 @@
       </c>
       <c r="C76" t="s">
         <v>1300</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CONTROLS_TITLE</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>HOTKEY_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>H: Controls</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>H：操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>HOTKEY_BATTLE</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Battle — Q: Retreat; C: Critical hit; Z/X: Attack/defense skill</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>战斗：Q 撤退，C 会心一击，Z/X 攻击/防御技能</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>GAMEPAD_MOVE</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Left stick / D-pad: Move</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>左摇杆／十字键：移动</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>GAMEPAD_MENU</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Menu: Open menu</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>菜单键：打开菜单</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>GAMEPAD_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>X: Controls</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>X：操作说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>GAMEPAD_CONFIRM</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>A: Confirm; B: Back</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>A：确认；B：返回</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>GAMEPAD_BATTLE</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Battle — B: Retreat; A: Critical hit; D-pad left/right: Attack/defense skill</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>战斗：B 撤退，A 会心一击，十字键左/右使用攻击/防御技能</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>TOUCH_MOVE</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Tap the map: Move to the destination</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>点击地图：移动到目标位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>TOUCH_MENU</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Tap an avatar: Menu; swipe avatars: Switch party member</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>点击头像：菜单；左右滑动头像：切换角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TOUCH_CONTROLS</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Tap Controls to view the controls</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>点击操作说明查看操作方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TOUCH_BATTLE</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Battle: Tap the skill, critical hit or retreat button</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>战斗：点击技能、会心一击或撤退按钮</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8059,7 +8269,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4933D5-C722-C646-96A3-51CA5B4C6607}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="43" customWidth="1"/>
@@ -8111,14 +8321,20 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>1199</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1265</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>1266</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TM_04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Press H to view the controls.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>按 H 键可以查看操作说明。</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -8174,6 +8390,74 @@
       </c>
       <c r="C10" s="2" t="s">
         <v>1458</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TM_04_G</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Press X to view the controls.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>按 X 键可以查看操作说明。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TM_04_M</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tap Controls to view the controls.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>点击操作说明可以查看操作方式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TM_05_G</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Enemy information. Press A to view details.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>敌人的能力信息，按 A 查看详细内容。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TM_07_MENU</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Open Items from the menu to use this item.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>打开菜单中的道具来使用。</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8565,6 +8849,40 @@
         <ns0:v>传送点</ns0:v>
       </ns0:c>
     </ns0:row>
+    <ns0:row r="35">
+      <ns0:c r="A35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MESSAGES_GAMEPAD_HOTKEY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Y: Leave a message</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Y：留言</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36">
+      <ns0:c r="A36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>MESSAGES_TOUCH_HOTKEY</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hold your current tile: Leave a message</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>长按角色当前格子：留言</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
   </ns0:sheetData>
   <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </ns0:worksheet>

</xml_diff>

<commit_message>
Sync with latest engine
</commit_message>
<xml_diff>
--- a/Data/Locale/Locale.xlsx
+++ b/Data/Locale/Locale.xlsx
@@ -5593,7 +5593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.33203125" customWidth="1"/>
@@ -6688,6 +6688,23 @@
       </c>
       <c r="C99" t="s">
         <v>1611</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>HOTKEY_SHOP_RECORDS</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>V: Visited shops</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>V：已访问商店</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>